<commit_message>
Update BIM and construction dashboard features
</commit_message>
<xml_diff>
--- a/public/data/정수처리시설_공정표.xlsx
+++ b/public/data/정수처리시설_공정표.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\126365_KH\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7A7F895-1FEB-4E97-A0C0-00D619439E0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF8D771A-D31E-4570-BAD6-326548223B0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="162">
   <si>
     <t>구분</t>
   </si>
@@ -534,6 +534,18 @@
   </si>
   <si>
     <t>임시 예정공정표</t>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <t>2025-06</t>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <t>2025-09</t>
+    <phoneticPr fontId="11" type="noConversion"/>
+  </si>
+  <si>
+    <t>2025-11</t>
     <phoneticPr fontId="11" type="noConversion"/>
   </si>
 </sst>
@@ -772,7 +784,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -797,22 +809,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -828,18 +825,34 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -1142,35 +1155,35 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="5" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="60" customWidth="1"/>
-    <col min="5" max="6" width="10" style="21" customWidth="1"/>
+    <col min="5" max="6" width="10" style="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="27" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="28"/>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-    </row>
-    <row r="3" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="23"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+    </row>
+    <row r="3" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -1183,618 +1196,619 @@
       <c r="D3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="20" t="s">
+      <c r="E3" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="20" t="s">
+      <c r="F3" s="11" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="22" t="s">
+    <row r="4" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="B4" s="22">
+      <c r="B4" s="13">
         <v>1</v>
       </c>
-      <c r="C4" s="29" t="s">
+      <c r="C4" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="29" t="s">
+      <c r="D4" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="30" t="s">
+      <c r="E4" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="30" t="s">
+      <c r="F4" s="19" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="22" t="s">
+    <row r="5" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="B5" s="22">
+      <c r="B5" s="13">
         <v>2</v>
       </c>
-      <c r="C5" s="29" t="s">
+      <c r="C5" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="30" t="s">
+      <c r="E5" s="19" t="s">
+        <v>159</v>
+      </c>
+      <c r="F5" s="19" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="B6" s="13">
+        <v>2</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="F6" s="19" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="B7" s="13">
+        <v>3</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" s="19" t="s">
+        <v>129</v>
+      </c>
+      <c r="F7" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="J7" s="10"/>
+    </row>
+    <row r="8" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="B8" s="13">
+        <v>4</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="19" t="s">
+        <v>132</v>
+      </c>
+      <c r="F8" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="F5" s="30" t="s">
+    </row>
+    <row r="9" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="B9" s="13">
+        <v>5</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="F9" s="19" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="13">
+        <v>6</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="19" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="13">
+        <v>7</v>
+      </c>
+      <c r="C11" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="E11" s="19" t="s">
+        <v>135</v>
+      </c>
+      <c r="F11" s="19" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="22" t="s">
-        <v>134</v>
-      </c>
-      <c r="B6" s="22">
-        <v>2</v>
-      </c>
-      <c r="C6" s="29" t="s">
+    <row r="12" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="13">
+        <v>8</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="E12" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="F12" s="19" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="13">
+        <v>9</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="E13" s="19" t="s">
+        <v>135</v>
+      </c>
+      <c r="F13" s="19" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" s="13">
+        <v>10</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="E14" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="F14" s="19" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="13">
+        <v>11</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="E15" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="F15" s="19" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" s="13">
         <v>12</v>
       </c>
-      <c r="D6" s="29" t="s">
+      <c r="C16" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="E16" s="19" t="s">
+        <v>142</v>
+      </c>
+      <c r="F16" s="19" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" s="13">
+        <v>13</v>
+      </c>
+      <c r="C17" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="E17" s="19" t="s">
+        <v>144</v>
+      </c>
+      <c r="F17" s="19" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" s="13">
+        <v>14</v>
+      </c>
+      <c r="C18" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="D18" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="E18" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="F18" s="19" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" s="13">
         <v>15</v>
       </c>
-      <c r="E6" s="30" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" s="30" t="s">
+      <c r="C19" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="D19" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="E19" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="F19" s="19" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" s="13">
         <v>16</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="22" t="s">
-        <v>134</v>
-      </c>
-      <c r="B7" s="22">
-        <v>3</v>
-      </c>
-      <c r="C7" s="29" t="s">
+      <c r="C20" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="D20" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="E20" s="19" t="s">
+        <v>148</v>
+      </c>
+      <c r="F20" s="19" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" s="13">
         <v>17</v>
       </c>
-      <c r="D7" s="29" t="s">
+      <c r="C21" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="D21" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="E21" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="F21" s="19" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B22" s="13">
         <v>18</v>
       </c>
-      <c r="E7" s="30" t="s">
-        <v>129</v>
-      </c>
-      <c r="F7" s="30" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="22" t="s">
-        <v>134</v>
-      </c>
-      <c r="B8" s="22">
-        <v>4</v>
-      </c>
-      <c r="C8" s="29" t="s">
-        <v>131</v>
-      </c>
-      <c r="D8" s="29" t="s">
+      <c r="C22" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="D22" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="E22" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="F22" s="19" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" s="13">
+        <v>19</v>
+      </c>
+      <c r="C23" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="D23" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="E23" s="19" t="s">
+        <v>150</v>
+      </c>
+      <c r="F23" s="19" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B24" s="13">
         <v>20</v>
       </c>
-      <c r="E8" s="30" t="s">
-        <v>132</v>
-      </c>
-      <c r="F8" s="30" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="22" t="s">
-        <v>134</v>
-      </c>
-      <c r="B9" s="22">
-        <v>5</v>
-      </c>
-      <c r="C9" s="29" t="s">
+      <c r="C24" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="D24" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="E24" s="19" t="s">
+        <v>151</v>
+      </c>
+      <c r="F24" s="19" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B25" s="13">
+        <v>21</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="D25" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="E25" s="19" t="s">
+        <v>142</v>
+      </c>
+      <c r="F25" s="19" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" s="13">
         <v>22</v>
       </c>
-      <c r="D9" s="29" t="s">
+      <c r="C26" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="D26" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="E26" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="F26" s="19" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B27" s="13">
         <v>23</v>
       </c>
-      <c r="E9" s="30" t="s">
+      <c r="C27" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="D27" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="E27" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="F27" s="19" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B28" s="13">
         <v>24</v>
       </c>
-      <c r="F9" s="30" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B10" s="22">
-        <v>6</v>
-      </c>
-      <c r="C10" s="29" t="s">
+      <c r="C28" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="D28" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="E28" s="19" t="s">
+        <v>154</v>
+      </c>
+      <c r="F28" s="19" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B29" s="13">
+        <v>25</v>
+      </c>
+      <c r="C29" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="D29" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="E29" s="19" t="s">
+        <v>148</v>
+      </c>
+      <c r="F29" s="19" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B30" s="13">
         <v>26</v>
       </c>
-      <c r="D10" s="29" t="s">
+      <c r="C30" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="D30" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="E30" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="F30" s="19" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B31" s="13">
+        <v>27</v>
+      </c>
+      <c r="C31" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="D31" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="E31" s="19" t="s">
+        <v>156</v>
+      </c>
+      <c r="F31" s="19" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B32" s="13">
         <v>28</v>
       </c>
-      <c r="E10" s="30" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="30" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" s="22">
-        <v>7</v>
-      </c>
-      <c r="C11" s="29" t="s">
-        <v>30</v>
-      </c>
-      <c r="D11" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="E11" s="30" t="s">
-        <v>135</v>
-      </c>
-      <c r="F11" s="30" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B12" s="22">
-        <v>8</v>
-      </c>
-      <c r="C12" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" s="29" t="s">
-        <v>33</v>
-      </c>
-      <c r="E12" s="30" t="s">
-        <v>136</v>
-      </c>
-      <c r="F12" s="30" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B13" s="22">
-        <v>9</v>
-      </c>
-      <c r="C13" s="29" t="s">
-        <v>34</v>
-      </c>
-      <c r="D13" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="E13" s="30" t="s">
-        <v>135</v>
-      </c>
-      <c r="F13" s="30" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B14" s="22">
-        <v>10</v>
-      </c>
-      <c r="C14" s="29" t="s">
-        <v>37</v>
-      </c>
-      <c r="D14" s="29" t="s">
-        <v>38</v>
-      </c>
-      <c r="E14" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="F14" s="30" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B15" s="22">
-        <v>11</v>
-      </c>
-      <c r="C15" s="29" t="s">
-        <v>139</v>
-      </c>
-      <c r="D15" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="E15" s="30" t="s">
-        <v>40</v>
-      </c>
-      <c r="F15" s="30" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B16" s="22">
-        <v>12</v>
-      </c>
-      <c r="C16" s="29" t="s">
-        <v>41</v>
-      </c>
-      <c r="D16" s="29" t="s">
-        <v>42</v>
-      </c>
-      <c r="E16" s="30" t="s">
-        <v>142</v>
-      </c>
-      <c r="F16" s="30" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B17" s="22">
-        <v>13</v>
-      </c>
-      <c r="C17" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="D17" s="29" t="s">
-        <v>45</v>
-      </c>
-      <c r="E17" s="30" t="s">
-        <v>144</v>
-      </c>
-      <c r="F17" s="30" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B18" s="22">
-        <v>14</v>
-      </c>
-      <c r="C18" s="29" t="s">
-        <v>46</v>
-      </c>
-      <c r="D18" s="29" t="s">
-        <v>47</v>
-      </c>
-      <c r="E18" s="30" t="s">
-        <v>146</v>
-      </c>
-      <c r="F18" s="30" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B19" s="22">
-        <v>15</v>
-      </c>
-      <c r="C19" s="29" t="s">
-        <v>48</v>
-      </c>
-      <c r="D19" s="29" t="s">
-        <v>49</v>
-      </c>
-      <c r="E19" s="30" t="s">
-        <v>50</v>
-      </c>
-      <c r="F19" s="30" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B20" s="22">
-        <v>16</v>
-      </c>
-      <c r="C20" s="29" t="s">
-        <v>52</v>
-      </c>
-      <c r="D20" s="29" t="s">
-        <v>53</v>
-      </c>
-      <c r="E20" s="30" t="s">
-        <v>148</v>
-      </c>
-      <c r="F20" s="30" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B21" s="22">
-        <v>17</v>
-      </c>
-      <c r="C21" s="29" t="s">
-        <v>54</v>
-      </c>
-      <c r="D21" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="E21" s="30" t="s">
-        <v>127</v>
-      </c>
-      <c r="F21" s="30" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B22" s="22">
-        <v>18</v>
-      </c>
-      <c r="C22" s="29" t="s">
-        <v>56</v>
-      </c>
-      <c r="D22" s="29" t="s">
-        <v>57</v>
-      </c>
-      <c r="E22" s="30" t="s">
-        <v>141</v>
-      </c>
-      <c r="F22" s="30" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B23" s="22">
-        <v>19</v>
-      </c>
-      <c r="C23" s="29" t="s">
-        <v>58</v>
-      </c>
-      <c r="D23" s="29" t="s">
-        <v>59</v>
-      </c>
-      <c r="E23" s="30" t="s">
-        <v>150</v>
-      </c>
-      <c r="F23" s="30" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B24" s="22">
-        <v>20</v>
-      </c>
-      <c r="C24" s="29" t="s">
-        <v>60</v>
-      </c>
-      <c r="D24" s="29" t="s">
-        <v>57</v>
-      </c>
-      <c r="E24" s="30" t="s">
-        <v>151</v>
-      </c>
-      <c r="F24" s="30" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B25" s="22">
-        <v>21</v>
-      </c>
-      <c r="C25" s="29" t="s">
-        <v>61</v>
-      </c>
-      <c r="D25" s="29" t="s">
-        <v>62</v>
-      </c>
-      <c r="E25" s="30" t="s">
-        <v>142</v>
-      </c>
-      <c r="F25" s="30" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B26" s="22">
-        <v>22</v>
-      </c>
-      <c r="C26" s="29" t="s">
-        <v>63</v>
-      </c>
-      <c r="D26" s="29" t="s">
-        <v>57</v>
-      </c>
-      <c r="E26" s="30" t="s">
-        <v>152</v>
-      </c>
-      <c r="F26" s="30" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B27" s="22">
-        <v>23</v>
-      </c>
-      <c r="C27" s="29" t="s">
-        <v>64</v>
-      </c>
-      <c r="D27" s="29" t="s">
-        <v>65</v>
-      </c>
-      <c r="E27" s="30" t="s">
-        <v>153</v>
-      </c>
-      <c r="F27" s="30" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B28" s="22">
-        <v>24</v>
-      </c>
-      <c r="C28" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="D28" s="29" t="s">
-        <v>67</v>
-      </c>
-      <c r="E28" s="30" t="s">
-        <v>154</v>
-      </c>
-      <c r="F28" s="30" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B29" s="22">
-        <v>25</v>
-      </c>
-      <c r="C29" s="29" t="s">
-        <v>69</v>
-      </c>
-      <c r="D29" s="29" t="s">
-        <v>70</v>
-      </c>
-      <c r="E29" s="30" t="s">
-        <v>148</v>
-      </c>
-      <c r="F29" s="30" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B30" s="22">
-        <v>26</v>
-      </c>
-      <c r="C30" s="29" t="s">
-        <v>71</v>
-      </c>
-      <c r="D30" s="29" t="s">
-        <v>72</v>
-      </c>
-      <c r="E30" s="30" t="s">
-        <v>141</v>
-      </c>
-      <c r="F30" s="30" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B31" s="22">
-        <v>27</v>
-      </c>
-      <c r="C31" s="29" t="s">
-        <v>73</v>
-      </c>
-      <c r="D31" s="29" t="s">
-        <v>74</v>
-      </c>
-      <c r="E31" s="30" t="s">
-        <v>156</v>
-      </c>
-      <c r="F31" s="30" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B32" s="22">
-        <v>28</v>
-      </c>
-      <c r="C32" s="29" t="s">
+      <c r="C32" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="D32" s="29" t="s">
+      <c r="D32" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="E32" s="30" t="s">
+      <c r="E32" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="F32" s="30" t="s">
+      <c r="F32" s="19" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="10"/>
-      <c r="B34" s="11"/>
-      <c r="C34" s="11"/>
-      <c r="D34" s="11"/>
-      <c r="E34" s="11"/>
-      <c r="F34" s="11"/>
+      <c r="A34" s="20"/>
+      <c r="B34" s="21"/>
+      <c r="C34" s="21"/>
+      <c r="D34" s="21"/>
+      <c r="E34" s="21"/>
+      <c r="F34" s="21"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="23"/>
-      <c r="B36" s="24"/>
-      <c r="C36" s="25"/>
-      <c r="D36" s="26"/>
+      <c r="A36" s="14"/>
+      <c r="B36" s="15"/>
+      <c r="C36" s="16"/>
+      <c r="D36" s="17"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="26"/>
-      <c r="B37" s="26"/>
-      <c r="C37" s="26"/>
-      <c r="D37" s="26"/>
+      <c r="A37" s="17"/>
+      <c r="B37" s="17"/>
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="26"/>
-      <c r="B38" s="26"/>
-      <c r="C38" s="26"/>
-      <c r="D38" s="26"/>
+      <c r="A38" s="17"/>
+      <c r="B38" s="17"/>
+      <c r="C38" s="17"/>
+      <c r="D38" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1819,66 +1833,66 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:58" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
-      <c r="L1" s="11"/>
-      <c r="M1" s="11"/>
-      <c r="N1" s="11"/>
-      <c r="O1" s="11"/>
-      <c r="P1" s="11"/>
-      <c r="Q1" s="11"/>
-      <c r="R1" s="11"/>
-      <c r="S1" s="11"/>
-      <c r="T1" s="11"/>
-      <c r="U1" s="11"/>
-      <c r="V1" s="11"/>
-      <c r="W1" s="11"/>
-      <c r="X1" s="11"/>
-      <c r="Y1" s="11"/>
-      <c r="Z1" s="11"/>
-      <c r="AA1" s="11"/>
-      <c r="AB1" s="11"/>
-      <c r="AC1" s="11"/>
-      <c r="AD1" s="11"/>
-      <c r="AE1" s="11"/>
-      <c r="AF1" s="11"/>
-      <c r="AG1" s="11"/>
-      <c r="AH1" s="11"/>
-      <c r="AI1" s="11"/>
-      <c r="AJ1" s="11"/>
-      <c r="AK1" s="11"/>
-      <c r="AL1" s="11"/>
-      <c r="AM1" s="11"/>
-      <c r="AN1" s="11"/>
-      <c r="AO1" s="11"/>
-      <c r="AP1" s="11"/>
-      <c r="AQ1" s="11"/>
-      <c r="AR1" s="11"/>
-      <c r="AS1" s="11"/>
-      <c r="AT1" s="11"/>
-      <c r="AU1" s="11"/>
-      <c r="AV1" s="11"/>
-      <c r="AW1" s="11"/>
-      <c r="AX1" s="11"/>
-      <c r="AY1" s="11"/>
-      <c r="AZ1" s="11"/>
-      <c r="BA1" s="11"/>
-      <c r="BB1" s="11"/>
-      <c r="BC1" s="11"/>
-      <c r="BD1" s="11"/>
-      <c r="BE1" s="11"/>
-      <c r="BF1" s="11"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="21"/>
+      <c r="O1" s="21"/>
+      <c r="P1" s="21"/>
+      <c r="Q1" s="21"/>
+      <c r="R1" s="21"/>
+      <c r="S1" s="21"/>
+      <c r="T1" s="21"/>
+      <c r="U1" s="21"/>
+      <c r="V1" s="21"/>
+      <c r="W1" s="21"/>
+      <c r="X1" s="21"/>
+      <c r="Y1" s="21"/>
+      <c r="Z1" s="21"/>
+      <c r="AA1" s="21"/>
+      <c r="AB1" s="21"/>
+      <c r="AC1" s="21"/>
+      <c r="AD1" s="21"/>
+      <c r="AE1" s="21"/>
+      <c r="AF1" s="21"/>
+      <c r="AG1" s="21"/>
+      <c r="AH1" s="21"/>
+      <c r="AI1" s="21"/>
+      <c r="AJ1" s="21"/>
+      <c r="AK1" s="21"/>
+      <c r="AL1" s="21"/>
+      <c r="AM1" s="21"/>
+      <c r="AN1" s="21"/>
+      <c r="AO1" s="21"/>
+      <c r="AP1" s="21"/>
+      <c r="AQ1" s="21"/>
+      <c r="AR1" s="21"/>
+      <c r="AS1" s="21"/>
+      <c r="AT1" s="21"/>
+      <c r="AU1" s="21"/>
+      <c r="AV1" s="21"/>
+      <c r="AW1" s="21"/>
+      <c r="AX1" s="21"/>
+      <c r="AY1" s="21"/>
+      <c r="AZ1" s="21"/>
+      <c r="BA1" s="21"/>
+      <c r="BB1" s="21"/>
+      <c r="BC1" s="21"/>
+      <c r="BD1" s="21"/>
+      <c r="BE1" s="21"/>
+      <c r="BF1" s="21"/>
     </row>
     <row r="2" spans="1:58" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -1889,96 +1903,96 @@
       </c>
     </row>
     <row r="3" spans="1:58" x14ac:dyDescent="0.3">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="D3" s="29" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:58" ht="27" x14ac:dyDescent="0.3">
-      <c r="A4" s="17"/>
-      <c r="B4" s="17"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
+      <c r="A4" s="30"/>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
       <c r="E4" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
-      <c r="I4" s="14"/>
-      <c r="J4" s="14"/>
-      <c r="K4" s="14"/>
-      <c r="L4" s="14"/>
-      <c r="M4" s="14"/>
-      <c r="N4" s="14"/>
-      <c r="O4" s="14"/>
-      <c r="P4" s="14"/>
-      <c r="Q4" s="15"/>
-      <c r="R4" s="13" t="s">
+      <c r="G4" s="26"/>
+      <c r="H4" s="26"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="26"/>
+      <c r="K4" s="26"/>
+      <c r="L4" s="26"/>
+      <c r="M4" s="26"/>
+      <c r="N4" s="26"/>
+      <c r="O4" s="26"/>
+      <c r="P4" s="26"/>
+      <c r="Q4" s="27"/>
+      <c r="R4" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="S4" s="14"/>
-      <c r="T4" s="14"/>
-      <c r="U4" s="14"/>
-      <c r="V4" s="14"/>
-      <c r="W4" s="14"/>
-      <c r="X4" s="14"/>
-      <c r="Y4" s="14"/>
-      <c r="Z4" s="14"/>
-      <c r="AA4" s="14"/>
-      <c r="AB4" s="14"/>
-      <c r="AC4" s="15"/>
-      <c r="AD4" s="13" t="s">
+      <c r="S4" s="26"/>
+      <c r="T4" s="26"/>
+      <c r="U4" s="26"/>
+      <c r="V4" s="26"/>
+      <c r="W4" s="26"/>
+      <c r="X4" s="26"/>
+      <c r="Y4" s="26"/>
+      <c r="Z4" s="26"/>
+      <c r="AA4" s="26"/>
+      <c r="AB4" s="26"/>
+      <c r="AC4" s="27"/>
+      <c r="AD4" s="25" t="s">
         <v>81</v>
       </c>
-      <c r="AE4" s="14"/>
-      <c r="AF4" s="14"/>
-      <c r="AG4" s="14"/>
-      <c r="AH4" s="14"/>
-      <c r="AI4" s="14"/>
-      <c r="AJ4" s="14"/>
-      <c r="AK4" s="14"/>
-      <c r="AL4" s="14"/>
-      <c r="AM4" s="14"/>
-      <c r="AN4" s="14"/>
-      <c r="AO4" s="15"/>
-      <c r="AP4" s="13" t="s">
+      <c r="AE4" s="26"/>
+      <c r="AF4" s="26"/>
+      <c r="AG4" s="26"/>
+      <c r="AH4" s="26"/>
+      <c r="AI4" s="26"/>
+      <c r="AJ4" s="26"/>
+      <c r="AK4" s="26"/>
+      <c r="AL4" s="26"/>
+      <c r="AM4" s="26"/>
+      <c r="AN4" s="26"/>
+      <c r="AO4" s="27"/>
+      <c r="AP4" s="25" t="s">
         <v>82</v>
       </c>
-      <c r="AQ4" s="14"/>
-      <c r="AR4" s="14"/>
-      <c r="AS4" s="14"/>
-      <c r="AT4" s="14"/>
-      <c r="AU4" s="14"/>
-      <c r="AV4" s="14"/>
-      <c r="AW4" s="14"/>
-      <c r="AX4" s="14"/>
-      <c r="AY4" s="14"/>
-      <c r="AZ4" s="14"/>
-      <c r="BA4" s="15"/>
-      <c r="BB4" s="13" t="s">
+      <c r="AQ4" s="26"/>
+      <c r="AR4" s="26"/>
+      <c r="AS4" s="26"/>
+      <c r="AT4" s="26"/>
+      <c r="AU4" s="26"/>
+      <c r="AV4" s="26"/>
+      <c r="AW4" s="26"/>
+      <c r="AX4" s="26"/>
+      <c r="AY4" s="26"/>
+      <c r="AZ4" s="26"/>
+      <c r="BA4" s="27"/>
+      <c r="BB4" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="BC4" s="14"/>
-      <c r="BD4" s="14"/>
-      <c r="BE4" s="14"/>
-      <c r="BF4" s="15"/>
+      <c r="BC4" s="26"/>
+      <c r="BD4" s="26"/>
+      <c r="BE4" s="26"/>
+      <c r="BF4" s="27"/>
     </row>
     <row r="5" spans="1:58" x14ac:dyDescent="0.3">
-      <c r="A5" s="18"/>
-      <c r="B5" s="18"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
+      <c r="A5" s="31"/>
+      <c r="B5" s="31"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="31"/>
       <c r="E5" s="5">
         <v>12</v>
       </c>
@@ -3238,18 +3252,18 @@
       <c r="BD46" s="9"/>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A49" s="19" t="s">
+      <c r="A49" s="24" t="s">
         <v>126</v>
       </c>
-      <c r="B49" s="11"/>
-      <c r="C49" s="11"/>
-      <c r="D49" s="11"/>
-      <c r="E49" s="11"/>
-      <c r="F49" s="11"/>
-      <c r="G49" s="11"/>
-      <c r="H49" s="11"/>
-      <c r="I49" s="11"/>
-      <c r="J49" s="11"/>
+      <c r="B49" s="21"/>
+      <c r="C49" s="21"/>
+      <c r="D49" s="21"/>
+      <c r="E49" s="21"/>
+      <c r="F49" s="21"/>
+      <c r="G49" s="21"/>
+      <c r="H49" s="21"/>
+      <c r="I49" s="21"/>
+      <c r="J49" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="11">

</xml_diff>